<commit_message>
feat(data): add initail excel datasets for course notes
</commit_message>
<xml_diff>
--- a/data/excel-files/laptop-sales.xlsx
+++ b/data/excel-files/laptop-sales.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <si>
     <t xml:space="preserve">Year</t>
   </si>
@@ -49,19 +49,22 @@
     <t xml:space="preserve">Mouse</t>
   </si>
   <si>
+    <t xml:space="preserve"># Laptop Sales Report</t>
+  </si>
+  <si>
     <t xml:space="preserve">Keyboard</t>
   </si>
   <si>
     <t xml:space="preserve">Monitor</t>
   </si>
   <si>
-    <t xml:space="preserve">Dataset Info:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date of Generation: 2026-03-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generated By: Google Gemini</t>
+    <t xml:space="preserve"># Dataset Info:</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Date of Generation: 2026-03-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve"># Generated By: Google Gemini</t>
   </si>
 </sst>
 </file>
@@ -151,13 +154,21 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -352,125 +363,146 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.4"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="C2" s="0" t="n">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="0" t="n">
+      <c r="F2" s="1" t="n">
         <v>1200</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="C3" s="0" t="n">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="0" t="n">
+      <c r="F3" s="1" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="C4" s="0" t="n">
+      <c r="A4" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="E4" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="0" t="n">
+      <c r="E5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1" t="n">
         <v>75</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="C5" s="0" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="E5" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="0" t="n">
+      <c r="E6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="1" t="n">
         <v>300</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>11</v>
-      </c>
-    </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>